<commit_message>
Agregado punto 3 (A validar)
</commit_message>
<xml_diff>
--- a/Tablas de Caja Negra - TP Clinica .xlsx
+++ b/Tablas de Caja Negra - TP Clinica .xlsx
@@ -1,10 +1,11 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <sheets>
-    <sheet name="Setters" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Integración" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Setters" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Integración" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mocks y Concurrencia" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -4780,8 +4781,8 @@
     <mergeCell ref="A94:E94"/>
     <mergeCell ref="D22:E22"/>
     <mergeCell ref="B115:C115"/>
+    <mergeCell ref="B102:C102"/>
     <mergeCell ref="D36:E36"/>
-    <mergeCell ref="B102:C102"/>
     <mergeCell ref="D45:E45"/>
     <mergeCell ref="A6:H6"/>
     <mergeCell ref="B12:C12"/>
@@ -4919,4 +4920,2984 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H133"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="13.88" customWidth="1" style="43" min="1" max="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="54" t="inlineStr">
+        <is>
+          <t>Tabla de Particiones setState(State) con mock</t>
+        </is>
+      </c>
+      <c r="B1" s="45" t="n"/>
+      <c r="C1" s="45" t="n"/>
+      <c r="D1" s="45" t="n"/>
+      <c r="E1" s="46" t="n"/>
+    </row>
+    <row r="2">
+      <c r="A2" s="47" t="inlineStr">
+        <is>
+          <t>Condición</t>
+        </is>
+      </c>
+      <c r="B2" s="38" t="inlineStr">
+        <is>
+          <t>Clase correcta</t>
+        </is>
+      </c>
+      <c r="C2" s="38" t="inlineStr">
+        <is>
+          <t>Clase</t>
+        </is>
+      </c>
+      <c r="D2" s="38" t="inlineStr">
+        <is>
+          <t>Clase errónea</t>
+        </is>
+      </c>
+      <c r="E2" s="38" t="inlineStr">
+        <is>
+          <t>Clase</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="15" customHeight="1" s="43">
+      <c r="A3" s="47" t="inlineStr">
+        <is>
+          <t>nuevoEstado</t>
+        </is>
+      </c>
+      <c r="B3" s="38" t="inlineStr">
+        <is>
+          <t>!= null (mock de State)</t>
+        </is>
+      </c>
+      <c r="C3" s="38" t="n">
+        <v>1</v>
+      </c>
+      <c r="D3" s="38" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+      <c r="E3" s="38" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="47" t="inlineStr">
+        <is>
+          <t>Bateria de pruebas setState(State) con mock</t>
+        </is>
+      </c>
+      <c r="B5" s="45" t="n"/>
+      <c r="C5" s="45" t="n"/>
+      <c r="D5" s="45" t="n"/>
+      <c r="E5" s="45" t="n"/>
+      <c r="F5" s="45" t="n"/>
+      <c r="G5" s="45" t="n"/>
+      <c r="H5" s="46" t="n"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="47" t="n"/>
+      <c r="B6" s="38" t="inlineStr">
+        <is>
+          <t>Entrada</t>
+        </is>
+      </c>
+      <c r="C6" s="46" t="n"/>
+      <c r="D6" s="38" t="inlineStr">
+        <is>
+          <t>Salida</t>
+        </is>
+      </c>
+      <c r="E6" s="46" t="n"/>
+      <c r="F6" s="38" t="inlineStr">
+        <is>
+          <t>Clases cubiertas</t>
+        </is>
+      </c>
+      <c r="G6" s="38" t="inlineStr">
+        <is>
+          <t>Valores limite</t>
+        </is>
+      </c>
+      <c r="H6" s="38" t="inlineStr">
+        <is>
+          <t>Salidas</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="30" customHeight="1" s="43">
+      <c r="A7" s="47" t="inlineStr">
+        <is>
+          <t>Clases correctas</t>
+        </is>
+      </c>
+      <c r="B7" s="38" t="inlineStr">
+        <is>
+          <t>setState(mock)</t>
+        </is>
+      </c>
+      <c r="C7" s="46" t="n"/>
+      <c r="D7" s="38" t="inlineStr">
+        <is>
+          <t>getEstadoActual() devuelve el mismo mock</t>
+        </is>
+      </c>
+      <c r="E7" s="46" t="n"/>
+      <c r="F7" s="38" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="G7" s="38" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H7" s="38" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="15" customHeight="1" s="43">
+      <c r="A8" s="47" t="inlineStr">
+        <is>
+          <t>Clases erróneas</t>
+        </is>
+      </c>
+      <c r="B8" s="38" t="inlineStr">
+        <is>
+          <t>setState(null)</t>
+        </is>
+      </c>
+      <c r="C8" s="46" t="n"/>
+      <c r="D8" s="38" t="inlineStr">
+        <is>
+          <t>AssertionError</t>
+        </is>
+      </c>
+      <c r="E8" s="46" t="n"/>
+      <c r="F8" s="38" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="G8" s="38" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H8" s="38" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="54" t="inlineStr">
+        <is>
+          <t>Tabla de Particiones solicitarMantenimiento(operario) con mock de State</t>
+        </is>
+      </c>
+      <c r="B11" s="45" t="n"/>
+      <c r="C11" s="45" t="n"/>
+      <c r="D11" s="45" t="n"/>
+      <c r="E11" s="46" t="n"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="47" t="inlineStr">
+        <is>
+          <t>Condición</t>
+        </is>
+      </c>
+      <c r="B12" s="38" t="inlineStr">
+        <is>
+          <t>Clase correcta</t>
+        </is>
+      </c>
+      <c r="C12" s="38" t="inlineStr">
+        <is>
+          <t>Clase</t>
+        </is>
+      </c>
+      <c r="D12" s="38" t="inlineStr">
+        <is>
+          <t>Clase errónea</t>
+        </is>
+      </c>
+      <c r="E12" s="38" t="inlineStr">
+        <is>
+          <t>Clase</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="15" customHeight="1" s="43">
+      <c r="A13" s="47" t="inlineStr">
+        <is>
+          <t>operario</t>
+        </is>
+      </c>
+      <c r="B13" s="38" t="inlineStr">
+        <is>
+          <t>!= null</t>
+        </is>
+      </c>
+      <c r="C13" s="38" t="n">
+        <v>1</v>
+      </c>
+      <c r="D13" s="38" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+      <c r="E13" s="38" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="14" ht="15" customHeight="1" s="43">
+      <c r="A14" s="47" t="inlineStr">
+        <is>
+          <t>ambulancia</t>
+        </is>
+      </c>
+      <c r="B14" s="38" t="inlineStr">
+        <is>
+          <t>Libre (ocupado = false)</t>
+        </is>
+      </c>
+      <c r="C14" s="38" t="n">
+        <v>3</v>
+      </c>
+      <c r="D14" s="38" t="inlineStr">
+        <is>
+          <t>Ocupada (ocupado = true)</t>
+        </is>
+      </c>
+      <c r="E14" s="38" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="15" ht="15" customHeight="1" s="43">
+      <c r="A15" s="47" t="inlineStr">
+        <is>
+          <t>simulacion</t>
+        </is>
+      </c>
+      <c r="B15" s="38" t="inlineStr">
+        <is>
+          <t>Activa</t>
+        </is>
+      </c>
+      <c r="C15" s="38" t="n">
+        <v>5</v>
+      </c>
+      <c r="D15" s="38" t="inlineStr">
+        <is>
+          <t>Finalizada</t>
+        </is>
+      </c>
+      <c r="E15" s="38" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="47" t="inlineStr">
+        <is>
+          <t>Bateria de pruebas solicitarMantenimiento(operario) con mock de State</t>
+        </is>
+      </c>
+      <c r="B17" s="45" t="n"/>
+      <c r="C17" s="45" t="n"/>
+      <c r="D17" s="45" t="n"/>
+      <c r="E17" s="45" t="n"/>
+      <c r="F17" s="45" t="n"/>
+      <c r="G17" s="45" t="n"/>
+      <c r="H17" s="46" t="n"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="47" t="n"/>
+      <c r="B18" s="38" t="inlineStr">
+        <is>
+          <t>Entrada</t>
+        </is>
+      </c>
+      <c r="C18" s="46" t="n"/>
+      <c r="D18" s="38" t="inlineStr">
+        <is>
+          <t>Salida</t>
+        </is>
+      </c>
+      <c r="E18" s="46" t="n"/>
+      <c r="F18" s="38" t="inlineStr">
+        <is>
+          <t>Clases cubiertas</t>
+        </is>
+      </c>
+      <c r="G18" s="38" t="inlineStr">
+        <is>
+          <t>Valores limite</t>
+        </is>
+      </c>
+      <c r="H18" s="38" t="inlineStr">
+        <is>
+          <t>Salidas</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="45" customHeight="1" s="43">
+      <c r="A19" s="47" t="inlineStr">
+        <is>
+          <t>Clases correctas</t>
+        </is>
+      </c>
+      <c r="B19" s="38" t="inlineStr">
+        <is>
+          <t>Operario valido, ambulancia libre, simulacion activa, estado = mock</t>
+        </is>
+      </c>
+      <c r="C19" s="46" t="n"/>
+      <c r="D19" s="38" t="inlineStr">
+        <is>
+          <t>El mock recibe SolicitudMantenimiento() una sola vez; ocupado = true</t>
+        </is>
+      </c>
+      <c r="E19" s="46" t="n"/>
+      <c r="F19" s="38" t="inlineStr">
+        <is>
+          <t>1, 3, 5</t>
+        </is>
+      </c>
+      <c r="G19" s="38" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H19" s="38" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="15" customHeight="1" s="43">
+      <c r="A20" s="47" t="inlineStr">
+        <is>
+          <t>Clases erróneas</t>
+        </is>
+      </c>
+      <c r="B20" s="38" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+      <c r="C20" s="46" t="n"/>
+      <c r="D20" s="38" t="inlineStr">
+        <is>
+          <t>AssertionError</t>
+        </is>
+      </c>
+      <c r="E20" s="46" t="n"/>
+      <c r="F20" s="38" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="G20" s="38" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H20" s="38" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="120" customHeight="1" s="43">
+      <c r="A21" s="55" t="n"/>
+      <c r="B21" s="38" t="inlineStr">
+        <is>
+          <t>Operario valido, ambulancia ocupada, simulacion activa (se llama desde un hilo aparte)</t>
+        </is>
+      </c>
+      <c r="C21" s="46" t="n"/>
+      <c r="D21" s="38" t="inlineStr">
+        <is>
+          <t>El hilo queda esperando (WAITING) y el mock no recibe ninguna llamada; al liberar la ambulancia con regresarSinPaciente() el hilo continua y el mock recibe SolicitudMantenimiento() una vez</t>
+        </is>
+      </c>
+      <c r="E21" s="46" t="n"/>
+      <c r="F21" s="38" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="G21" s="38" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H21" s="38" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="60" customHeight="1" s="43">
+      <c r="A22" s="50" t="n"/>
+      <c r="B22" s="38" t="inlineStr">
+        <is>
+          <t>Operario valido, simulacion finalizada (setSimulacionActiva(false))</t>
+        </is>
+      </c>
+      <c r="C22" s="46" t="n"/>
+      <c r="D22" s="38" t="inlineStr">
+        <is>
+          <t>Retorna sin esperar y sin llamar al estado: el mock no recibe ninguna llamada; ocupado sigue en false</t>
+        </is>
+      </c>
+      <c r="E22" s="46" t="n"/>
+      <c r="F22" s="38" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="G22" s="38" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H22" s="38" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="54" t="inlineStr">
+        <is>
+          <t>Tabla de Particiones atenderDomicilio(asociado) con mock de State</t>
+        </is>
+      </c>
+      <c r="B25" s="45" t="n"/>
+      <c r="C25" s="45" t="n"/>
+      <c r="D25" s="45" t="n"/>
+      <c r="E25" s="46" t="n"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="47" t="inlineStr">
+        <is>
+          <t>Condición</t>
+        </is>
+      </c>
+      <c r="B26" s="38" t="inlineStr">
+        <is>
+          <t>Clase correcta</t>
+        </is>
+      </c>
+      <c r="C26" s="38" t="inlineStr">
+        <is>
+          <t>Clase</t>
+        </is>
+      </c>
+      <c r="D26" s="38" t="inlineStr">
+        <is>
+          <t>Clase errónea</t>
+        </is>
+      </c>
+      <c r="E26" s="38" t="inlineStr">
+        <is>
+          <t>Clase</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="15" customHeight="1" s="43">
+      <c r="A27" s="47" t="inlineStr">
+        <is>
+          <t>asociado</t>
+        </is>
+      </c>
+      <c r="B27" s="38" t="inlineStr">
+        <is>
+          <t>!= null</t>
+        </is>
+      </c>
+      <c r="C27" s="38" t="n">
+        <v>1</v>
+      </c>
+      <c r="D27" s="38" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+      <c r="E27" s="38" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="28" ht="15" customHeight="1" s="43">
+      <c r="A28" s="47" t="inlineStr">
+        <is>
+          <t>ambulancia</t>
+        </is>
+      </c>
+      <c r="B28" s="38" t="inlineStr">
+        <is>
+          <t>Libre (ocupado = false)</t>
+        </is>
+      </c>
+      <c r="C28" s="38" t="n">
+        <v>3</v>
+      </c>
+      <c r="D28" s="38" t="inlineStr">
+        <is>
+          <t>Ocupada (ocupado = true)</t>
+        </is>
+      </c>
+      <c r="E28" s="38" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="29" ht="15" customHeight="1" s="43">
+      <c r="A29" s="47" t="inlineStr">
+        <is>
+          <t>simulacion</t>
+        </is>
+      </c>
+      <c r="B29" s="38" t="inlineStr">
+        <is>
+          <t>Activa</t>
+        </is>
+      </c>
+      <c r="C29" s="38" t="n">
+        <v>5</v>
+      </c>
+      <c r="D29" s="38" t="inlineStr">
+        <is>
+          <t>Finalizada</t>
+        </is>
+      </c>
+      <c r="E29" s="38" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="47" t="inlineStr">
+        <is>
+          <t>Bateria de pruebas atenderDomicilio(asociado) con mock de State</t>
+        </is>
+      </c>
+      <c r="B31" s="45" t="n"/>
+      <c r="C31" s="45" t="n"/>
+      <c r="D31" s="45" t="n"/>
+      <c r="E31" s="45" t="n"/>
+      <c r="F31" s="45" t="n"/>
+      <c r="G31" s="45" t="n"/>
+      <c r="H31" s="46" t="n"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="47" t="n"/>
+      <c r="B32" s="38" t="inlineStr">
+        <is>
+          <t>Entrada</t>
+        </is>
+      </c>
+      <c r="C32" s="46" t="n"/>
+      <c r="D32" s="38" t="inlineStr">
+        <is>
+          <t>Salida</t>
+        </is>
+      </c>
+      <c r="E32" s="46" t="n"/>
+      <c r="F32" s="38" t="inlineStr">
+        <is>
+          <t>Clases cubiertas</t>
+        </is>
+      </c>
+      <c r="G32" s="38" t="inlineStr">
+        <is>
+          <t>Valores limite</t>
+        </is>
+      </c>
+      <c r="H32" s="38" t="inlineStr">
+        <is>
+          <t>Salidas</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="45" customHeight="1" s="43">
+      <c r="A33" s="47" t="inlineStr">
+        <is>
+          <t>Clases correctas</t>
+        </is>
+      </c>
+      <c r="B33" s="38" t="inlineStr">
+        <is>
+          <t>Asociado valido, ambulancia libre, simulacion activa, estado = mock</t>
+        </is>
+      </c>
+      <c r="C33" s="46" t="n"/>
+      <c r="D33" s="38" t="inlineStr">
+        <is>
+          <t>El mock recibe SolicitudDeAtencionDomicilio() una sola vez; ocupado = true</t>
+        </is>
+      </c>
+      <c r="E33" s="46" t="n"/>
+      <c r="F33" s="38" t="inlineStr">
+        <is>
+          <t>1, 3, 5</t>
+        </is>
+      </c>
+      <c r="G33" s="38" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H33" s="38" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="15" customHeight="1" s="43">
+      <c r="A34" s="47" t="inlineStr">
+        <is>
+          <t>Clases erróneas</t>
+        </is>
+      </c>
+      <c r="B34" s="38" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+      <c r="C34" s="46" t="n"/>
+      <c r="D34" s="38" t="inlineStr">
+        <is>
+          <t>AssertionError</t>
+        </is>
+      </c>
+      <c r="E34" s="46" t="n"/>
+      <c r="F34" s="38" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="G34" s="38" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H34" s="38" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="35" ht="120" customHeight="1" s="43">
+      <c r="A35" s="55" t="n"/>
+      <c r="B35" s="38" t="inlineStr">
+        <is>
+          <t>Asociado valido, ambulancia ocupada, simulacion activa (se llama desde un hilo aparte)</t>
+        </is>
+      </c>
+      <c r="C35" s="46" t="n"/>
+      <c r="D35" s="38" t="inlineStr">
+        <is>
+          <t>El hilo queda esperando (WAITING) y el mock no recibe ninguna llamada; al liberar la ambulancia con regresarSinPaciente() el hilo continua y el mock recibe SolicitudDeAtencionDomicilio() una vez</t>
+        </is>
+      </c>
+      <c r="E35" s="46" t="n"/>
+      <c r="F35" s="38" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="G35" s="38" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H35" s="38" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" ht="60" customHeight="1" s="43">
+      <c r="A36" s="50" t="n"/>
+      <c r="B36" s="38" t="inlineStr">
+        <is>
+          <t>Asociado valido, simulacion finalizada (setSimulacionActiva(false))</t>
+        </is>
+      </c>
+      <c r="C36" s="46" t="n"/>
+      <c r="D36" s="38" t="inlineStr">
+        <is>
+          <t>Retorna sin esperar y sin llamar al estado: el mock no recibe ninguna llamada; ocupado sigue en false</t>
+        </is>
+      </c>
+      <c r="E36" s="46" t="n"/>
+      <c r="F36" s="38" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="G36" s="38" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H36" s="38" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="54" t="inlineStr">
+        <is>
+          <t>Tabla de Particiones trasladarALaClinica(asociado) con mock de State</t>
+        </is>
+      </c>
+      <c r="B39" s="45" t="n"/>
+      <c r="C39" s="45" t="n"/>
+      <c r="D39" s="45" t="n"/>
+      <c r="E39" s="46" t="n"/>
+    </row>
+    <row r="40">
+      <c r="A40" s="47" t="inlineStr">
+        <is>
+          <t>Condición</t>
+        </is>
+      </c>
+      <c r="B40" s="38" t="inlineStr">
+        <is>
+          <t>Clase correcta</t>
+        </is>
+      </c>
+      <c r="C40" s="38" t="inlineStr">
+        <is>
+          <t>Clase</t>
+        </is>
+      </c>
+      <c r="D40" s="38" t="inlineStr">
+        <is>
+          <t>Clase errónea</t>
+        </is>
+      </c>
+      <c r="E40" s="38" t="inlineStr">
+        <is>
+          <t>Clase</t>
+        </is>
+      </c>
+    </row>
+    <row r="41" ht="15" customHeight="1" s="43">
+      <c r="A41" s="47" t="inlineStr">
+        <is>
+          <t>asociado</t>
+        </is>
+      </c>
+      <c r="B41" s="38" t="inlineStr">
+        <is>
+          <t>!= null</t>
+        </is>
+      </c>
+      <c r="C41" s="38" t="n">
+        <v>1</v>
+      </c>
+      <c r="D41" s="38" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+      <c r="E41" s="38" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="42" ht="15" customHeight="1" s="43">
+      <c r="A42" s="47" t="inlineStr">
+        <is>
+          <t>ambulancia</t>
+        </is>
+      </c>
+      <c r="B42" s="38" t="inlineStr">
+        <is>
+          <t>Libre (ocupado = false)</t>
+        </is>
+      </c>
+      <c r="C42" s="38" t="n">
+        <v>3</v>
+      </c>
+      <c r="D42" s="38" t="inlineStr">
+        <is>
+          <t>Ocupada (ocupado = true)</t>
+        </is>
+      </c>
+      <c r="E42" s="38" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="43" ht="15" customHeight="1" s="43">
+      <c r="A43" s="47" t="inlineStr">
+        <is>
+          <t>simulacion</t>
+        </is>
+      </c>
+      <c r="B43" s="38" t="inlineStr">
+        <is>
+          <t>Activa</t>
+        </is>
+      </c>
+      <c r="C43" s="38" t="n">
+        <v>5</v>
+      </c>
+      <c r="D43" s="38" t="inlineStr">
+        <is>
+          <t>Finalizada</t>
+        </is>
+      </c>
+      <c r="E43" s="38" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="47" t="inlineStr">
+        <is>
+          <t>Bateria de pruebas trasladarALaClinica(asociado) con mock de State</t>
+        </is>
+      </c>
+      <c r="B45" s="45" t="n"/>
+      <c r="C45" s="45" t="n"/>
+      <c r="D45" s="45" t="n"/>
+      <c r="E45" s="45" t="n"/>
+      <c r="F45" s="45" t="n"/>
+      <c r="G45" s="45" t="n"/>
+      <c r="H45" s="46" t="n"/>
+    </row>
+    <row r="46">
+      <c r="A46" s="47" t="n"/>
+      <c r="B46" s="38" t="inlineStr">
+        <is>
+          <t>Entrada</t>
+        </is>
+      </c>
+      <c r="C46" s="46" t="n"/>
+      <c r="D46" s="38" t="inlineStr">
+        <is>
+          <t>Salida</t>
+        </is>
+      </c>
+      <c r="E46" s="46" t="n"/>
+      <c r="F46" s="38" t="inlineStr">
+        <is>
+          <t>Clases cubiertas</t>
+        </is>
+      </c>
+      <c r="G46" s="38" t="inlineStr">
+        <is>
+          <t>Valores limite</t>
+        </is>
+      </c>
+      <c r="H46" s="38" t="inlineStr">
+        <is>
+          <t>Salidas</t>
+        </is>
+      </c>
+    </row>
+    <row r="47" ht="45" customHeight="1" s="43">
+      <c r="A47" s="47" t="inlineStr">
+        <is>
+          <t>Clases correctas</t>
+        </is>
+      </c>
+      <c r="B47" s="38" t="inlineStr">
+        <is>
+          <t>Asociado valido, ambulancia libre, simulacion activa, estado = mock</t>
+        </is>
+      </c>
+      <c r="C47" s="46" t="n"/>
+      <c r="D47" s="38" t="inlineStr">
+        <is>
+          <t>El mock recibe SolicitudDeTraslado() una sola vez; ocupado = true</t>
+        </is>
+      </c>
+      <c r="E47" s="46" t="n"/>
+      <c r="F47" s="38" t="inlineStr">
+        <is>
+          <t>1, 3, 5</t>
+        </is>
+      </c>
+      <c r="G47" s="38" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H47" s="38" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="48" ht="15" customHeight="1" s="43">
+      <c r="A48" s="47" t="inlineStr">
+        <is>
+          <t>Clases erróneas</t>
+        </is>
+      </c>
+      <c r="B48" s="38" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+      <c r="C48" s="46" t="n"/>
+      <c r="D48" s="38" t="inlineStr">
+        <is>
+          <t>AssertionError</t>
+        </is>
+      </c>
+      <c r="E48" s="46" t="n"/>
+      <c r="F48" s="38" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="G48" s="38" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H48" s="38" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="49" ht="120" customHeight="1" s="43">
+      <c r="A49" s="55" t="n"/>
+      <c r="B49" s="38" t="inlineStr">
+        <is>
+          <t>Asociado valido, ambulancia ocupada, simulacion activa (se llama desde un hilo aparte)</t>
+        </is>
+      </c>
+      <c r="C49" s="46" t="n"/>
+      <c r="D49" s="38" t="inlineStr">
+        <is>
+          <t>El hilo queda esperando (WAITING) y el mock no recibe ninguna llamada; al liberar la ambulancia con regresarSinPaciente() el hilo continua y el mock recibe SolicitudDeTraslado() una vez</t>
+        </is>
+      </c>
+      <c r="E49" s="46" t="n"/>
+      <c r="F49" s="38" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="G49" s="38" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H49" s="38" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="50" ht="60" customHeight="1" s="43">
+      <c r="A50" s="50" t="n"/>
+      <c r="B50" s="38" t="inlineStr">
+        <is>
+          <t>Asociado valido, simulacion finalizada (setSimulacionActiva(false))</t>
+        </is>
+      </c>
+      <c r="C50" s="46" t="n"/>
+      <c r="D50" s="38" t="inlineStr">
+        <is>
+          <t>Retorna sin esperar y sin llamar al estado: el mock no recibe ninguna llamada; ocupado sigue en false</t>
+        </is>
+      </c>
+      <c r="E50" s="46" t="n"/>
+      <c r="F50" s="38" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="G50" s="38" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H50" s="38" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="54" t="inlineStr">
+        <is>
+          <t>Tabla de Particiones Retornos y fin de mantenimiento con mock de State</t>
+        </is>
+      </c>
+      <c r="B53" s="45" t="n"/>
+      <c r="C53" s="45" t="n"/>
+      <c r="D53" s="45" t="n"/>
+      <c r="E53" s="46" t="n"/>
+    </row>
+    <row r="54">
+      <c r="A54" s="47" t="inlineStr">
+        <is>
+          <t>Condición</t>
+        </is>
+      </c>
+      <c r="B54" s="38" t="inlineStr">
+        <is>
+          <t>Clase correcta</t>
+        </is>
+      </c>
+      <c r="C54" s="38" t="inlineStr">
+        <is>
+          <t>Clase</t>
+        </is>
+      </c>
+      <c r="D54" s="38" t="inlineStr">
+        <is>
+          <t>Clase errónea</t>
+        </is>
+      </c>
+      <c r="E54" s="38" t="inlineStr">
+        <is>
+          <t>Clase</t>
+        </is>
+      </c>
+    </row>
+    <row r="55" ht="45" customHeight="1" s="43">
+      <c r="A55" s="47" t="inlineStr">
+        <is>
+          <t>operacion</t>
+        </is>
+      </c>
+      <c r="B55" s="38" t="inlineStr">
+        <is>
+          <t>retornoAutomatico, regresarSinPaciente o volviendoDelTaller</t>
+        </is>
+      </c>
+      <c r="C55" s="38" t="n">
+        <v>1</v>
+      </c>
+      <c r="D55" s="38" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E55" s="38" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="47" t="inlineStr">
+        <is>
+          <t>Bateria de pruebas Retornos y fin de mantenimiento con mock de State</t>
+        </is>
+      </c>
+      <c r="B57" s="45" t="n"/>
+      <c r="C57" s="45" t="n"/>
+      <c r="D57" s="45" t="n"/>
+      <c r="E57" s="45" t="n"/>
+      <c r="F57" s="45" t="n"/>
+      <c r="G57" s="45" t="n"/>
+      <c r="H57" s="46" t="n"/>
+    </row>
+    <row r="58">
+      <c r="A58" s="47" t="n"/>
+      <c r="B58" s="38" t="inlineStr">
+        <is>
+          <t>Entrada</t>
+        </is>
+      </c>
+      <c r="C58" s="46" t="n"/>
+      <c r="D58" s="38" t="inlineStr">
+        <is>
+          <t>Salida</t>
+        </is>
+      </c>
+      <c r="E58" s="46" t="n"/>
+      <c r="F58" s="38" t="inlineStr">
+        <is>
+          <t>Clases cubiertas</t>
+        </is>
+      </c>
+      <c r="G58" s="38" t="inlineStr">
+        <is>
+          <t>Valores limite</t>
+        </is>
+      </c>
+      <c r="H58" s="38" t="inlineStr">
+        <is>
+          <t>Salidas</t>
+        </is>
+      </c>
+    </row>
+    <row r="59" ht="30" customHeight="1" s="43">
+      <c r="A59" s="47" t="inlineStr">
+        <is>
+          <t>Clases correctas</t>
+        </is>
+      </c>
+      <c r="B59" s="38" t="inlineStr">
+        <is>
+          <t>retornoAutomatico(retorno) con estado = mock</t>
+        </is>
+      </c>
+      <c r="C59" s="46" t="n"/>
+      <c r="D59" s="38" t="inlineStr">
+        <is>
+          <t>El mock recibe RetornoClinica() una sola vez</t>
+        </is>
+      </c>
+      <c r="E59" s="46" t="n"/>
+      <c r="F59" s="38" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="G59" s="38" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H59" s="38" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="60" ht="45" customHeight="1" s="43">
+      <c r="A60" s="55" t="n"/>
+      <c r="B60" s="38" t="inlineStr">
+        <is>
+          <t>regresarSinPaciente() con ambulancia ocupada y estado = mock</t>
+        </is>
+      </c>
+      <c r="C60" s="46" t="n"/>
+      <c r="D60" s="38" t="inlineStr">
+        <is>
+          <t>El mock recibe RetornoClinica() una sola vez; ocupado = false</t>
+        </is>
+      </c>
+      <c r="E60" s="46" t="n"/>
+      <c r="F60" s="38" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="G60" s="38" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H60" s="38" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="61" ht="45" customHeight="1" s="43">
+      <c r="A61" s="50" t="n"/>
+      <c r="B61" s="38" t="inlineStr">
+        <is>
+          <t>volviendoDelTaller() con ambulancia ocupada y estado = mock</t>
+        </is>
+      </c>
+      <c r="C61" s="46" t="n"/>
+      <c r="D61" s="38" t="inlineStr">
+        <is>
+          <t>El mock recibe SolicitudMantenimiento() una sola vez; ocupado = false</t>
+        </is>
+      </c>
+      <c r="E61" s="46" t="n"/>
+      <c r="F61" s="38" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="G61" s="38" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H61" s="38" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="62" ht="15" customHeight="1" s="43">
+      <c r="A62" s="47" t="inlineStr">
+        <is>
+          <t>Clases erróneas</t>
+        </is>
+      </c>
+      <c r="B62" s="38" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="C62" s="46" t="n"/>
+      <c r="D62" s="38" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E62" s="46" t="n"/>
+      <c r="F62" s="38" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G62" s="38" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H62" s="38" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="54" t="inlineStr">
+        <is>
+          <t>Tabla de Particiones Transiciones de la maquina de estados (estados reales)</t>
+        </is>
+      </c>
+      <c r="B65" s="45" t="n"/>
+      <c r="C65" s="45" t="n"/>
+      <c r="D65" s="45" t="n"/>
+      <c r="E65" s="46" t="n"/>
+    </row>
+    <row r="66">
+      <c r="A66" s="47" t="inlineStr">
+        <is>
+          <t>Condición</t>
+        </is>
+      </c>
+      <c r="B66" s="38" t="inlineStr">
+        <is>
+          <t>Clase correcta</t>
+        </is>
+      </c>
+      <c r="C66" s="38" t="inlineStr">
+        <is>
+          <t>Clase</t>
+        </is>
+      </c>
+      <c r="D66" s="38" t="inlineStr">
+        <is>
+          <t>Clase errónea</t>
+        </is>
+      </c>
+      <c r="E66" s="38" t="inlineStr">
+        <is>
+          <t>Clase</t>
+        </is>
+      </c>
+    </row>
+    <row r="67" ht="15" customHeight="1" s="43">
+      <c r="A67" s="47" t="inlineStr">
+        <is>
+          <t>estado actual</t>
+        </is>
+      </c>
+      <c r="B67" s="38" t="inlineStr">
+        <is>
+          <t>Disponible</t>
+        </is>
+      </c>
+      <c r="C67" s="38" t="n">
+        <v>1</v>
+      </c>
+      <c r="D67" s="38" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E67" s="38" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="68" ht="30" customHeight="1" s="43">
+      <c r="A68" s="47" t="inlineStr">
+        <is>
+          <t>estado actual</t>
+        </is>
+      </c>
+      <c r="B68" s="38" t="inlineStr">
+        <is>
+          <t>Trasladando paciente a la clinica</t>
+        </is>
+      </c>
+      <c r="C68" s="38" t="n">
+        <v>2</v>
+      </c>
+      <c r="D68" s="38" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E68" s="38" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="69" ht="15" customHeight="1" s="43">
+      <c r="A69" s="47" t="inlineStr">
+        <is>
+          <t>estado actual</t>
+        </is>
+      </c>
+      <c r="B69" s="38" t="inlineStr">
+        <is>
+          <t>Atendiendo en domicilio</t>
+        </is>
+      </c>
+      <c r="C69" s="38" t="n">
+        <v>3</v>
+      </c>
+      <c r="D69" s="38" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E69" s="38" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="70" ht="30" customHeight="1" s="43">
+      <c r="A70" s="47" t="inlineStr">
+        <is>
+          <t>estado actual</t>
+        </is>
+      </c>
+      <c r="B70" s="38" t="inlineStr">
+        <is>
+          <t>Regresando a la clinica sin paciente</t>
+        </is>
+      </c>
+      <c r="C70" s="38" t="n">
+        <v>4</v>
+      </c>
+      <c r="D70" s="38" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E70" s="38" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="71" ht="15" customHeight="1" s="43">
+      <c r="A71" s="47" t="inlineStr">
+        <is>
+          <t>estado actual</t>
+        </is>
+      </c>
+      <c r="B71" s="38" t="inlineStr">
+        <is>
+          <t>En taller</t>
+        </is>
+      </c>
+      <c r="C71" s="38" t="n">
+        <v>5</v>
+      </c>
+      <c r="D71" s="38" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E71" s="38" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="72" ht="15" customHeight="1" s="43">
+      <c r="A72" s="47" t="inlineStr">
+        <is>
+          <t>estado actual</t>
+        </is>
+      </c>
+      <c r="B72" s="38" t="inlineStr">
+        <is>
+          <t>Regresando del taller</t>
+        </is>
+      </c>
+      <c r="C72" s="38" t="n">
+        <v>6</v>
+      </c>
+      <c r="D72" s="38" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E72" s="38" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="47" t="inlineStr">
+        <is>
+          <t>Bateria de pruebas Transiciones de la maquina de estados (estados reales)</t>
+        </is>
+      </c>
+      <c r="B74" s="45" t="n"/>
+      <c r="C74" s="45" t="n"/>
+      <c r="D74" s="45" t="n"/>
+      <c r="E74" s="45" t="n"/>
+      <c r="F74" s="45" t="n"/>
+      <c r="G74" s="45" t="n"/>
+      <c r="H74" s="46" t="n"/>
+    </row>
+    <row r="75">
+      <c r="A75" s="47" t="n"/>
+      <c r="B75" s="38" t="inlineStr">
+        <is>
+          <t>Entrada</t>
+        </is>
+      </c>
+      <c r="C75" s="46" t="n"/>
+      <c r="D75" s="38" t="inlineStr">
+        <is>
+          <t>Salida</t>
+        </is>
+      </c>
+      <c r="E75" s="46" t="n"/>
+      <c r="F75" s="38" t="inlineStr">
+        <is>
+          <t>Clases cubiertas</t>
+        </is>
+      </c>
+      <c r="G75" s="38" t="inlineStr">
+        <is>
+          <t>Valores limite</t>
+        </is>
+      </c>
+      <c r="H75" s="38" t="inlineStr">
+        <is>
+          <t>Salidas</t>
+        </is>
+      </c>
+    </row>
+    <row r="76" ht="30" customHeight="1" s="43">
+      <c r="A76" s="47" t="inlineStr">
+        <is>
+          <t>Clases correctas</t>
+        </is>
+      </c>
+      <c r="B76" s="38" t="inlineStr">
+        <is>
+          <t>Disponible + SolicitudDeTraslado()</t>
+        </is>
+      </c>
+      <c r="C76" s="46" t="n"/>
+      <c r="D76" s="38" t="inlineStr">
+        <is>
+          <t>Pasa a Trasladando paciente</t>
+        </is>
+      </c>
+      <c r="E76" s="46" t="n"/>
+      <c r="F76" s="38" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="G76" s="38" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H76" s="38" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="77" ht="30" customHeight="1" s="43">
+      <c r="A77" s="55" t="n"/>
+      <c r="B77" s="38" t="inlineStr">
+        <is>
+          <t>Disponible + SolicitudDeAtencionDomicilio()</t>
+        </is>
+      </c>
+      <c r="C77" s="46" t="n"/>
+      <c r="D77" s="38" t="inlineStr">
+        <is>
+          <t>Pasa a Atendiendo en domicilio</t>
+        </is>
+      </c>
+      <c r="E77" s="46" t="n"/>
+      <c r="F77" s="38" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="G77" s="38" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H77" s="38" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="78" ht="30" customHeight="1" s="43">
+      <c r="A78" s="55" t="n"/>
+      <c r="B78" s="38" t="inlineStr">
+        <is>
+          <t>Disponible + SolicitudMantenimiento()</t>
+        </is>
+      </c>
+      <c r="C78" s="46" t="n"/>
+      <c r="D78" s="38" t="inlineStr">
+        <is>
+          <t>Pasa a En taller</t>
+        </is>
+      </c>
+      <c r="E78" s="46" t="n"/>
+      <c r="F78" s="38" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="G78" s="38" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H78" s="38" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="79" ht="30" customHeight="1" s="43">
+      <c r="A79" s="55" t="n"/>
+      <c r="B79" s="38" t="inlineStr">
+        <is>
+          <t>Disponible + RetornoClinica()</t>
+        </is>
+      </c>
+      <c r="C79" s="46" t="n"/>
+      <c r="D79" s="38" t="inlineStr">
+        <is>
+          <t>Sigue en Disponible (ya esta en la clinica)</t>
+        </is>
+      </c>
+      <c r="E79" s="46" t="n"/>
+      <c r="F79" s="38" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="G79" s="38" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H79" s="38" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="80" ht="45" customHeight="1" s="43">
+      <c r="A80" s="55" t="n"/>
+      <c r="B80" s="38" t="inlineStr">
+        <is>
+          <t>Trasladando + RetornoClinica()</t>
+        </is>
+      </c>
+      <c r="C80" s="46" t="n"/>
+      <c r="D80" s="38" t="inlineStr">
+        <is>
+          <t>Pasa a Disponible (segun el Javadoc de la clase). Tarda 1 s por un sleep</t>
+        </is>
+      </c>
+      <c r="E80" s="46" t="n"/>
+      <c r="F80" s="38" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="G80" s="38" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H80" s="38" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="81" ht="30" customHeight="1" s="43">
+      <c r="A81" s="55" t="n"/>
+      <c r="B81" s="38" t="inlineStr">
+        <is>
+          <t>Trasladando + SolicitudDeTraslado()</t>
+        </is>
+      </c>
+      <c r="C81" s="46" t="n"/>
+      <c r="D81" s="38" t="inlineStr">
+        <is>
+          <t>Sigue en Trasladando (no puede atender)</t>
+        </is>
+      </c>
+      <c r="E81" s="46" t="n"/>
+      <c r="F81" s="38" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="G81" s="38" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H81" s="38" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="82" ht="30" customHeight="1" s="43">
+      <c r="A82" s="55" t="n"/>
+      <c r="B82" s="38" t="inlineStr">
+        <is>
+          <t>Atendiendo + RetornoClinica()</t>
+        </is>
+      </c>
+      <c r="C82" s="46" t="n"/>
+      <c r="D82" s="38" t="inlineStr">
+        <is>
+          <t>Pasa a Regresando sin paciente</t>
+        </is>
+      </c>
+      <c r="E82" s="46" t="n"/>
+      <c r="F82" s="38" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="G82" s="38" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H82" s="38" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="83" ht="30" customHeight="1" s="43">
+      <c r="A83" s="55" t="n"/>
+      <c r="B83" s="38" t="inlineStr">
+        <is>
+          <t>Atendiendo + SolicitudMantenimiento()</t>
+        </is>
+      </c>
+      <c r="C83" s="46" t="n"/>
+      <c r="D83" s="38" t="inlineStr">
+        <is>
+          <t>Sigue en Atendiendo (no puede atender)</t>
+        </is>
+      </c>
+      <c r="E83" s="46" t="n"/>
+      <c r="F83" s="38" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="G83" s="38" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H83" s="38" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="84" ht="30" customHeight="1" s="43">
+      <c r="A84" s="55" t="n"/>
+      <c r="B84" s="38" t="inlineStr">
+        <is>
+          <t>Regresando sin paciente + RetornoClinica()</t>
+        </is>
+      </c>
+      <c r="C84" s="46" t="n"/>
+      <c r="D84" s="38" t="inlineStr">
+        <is>
+          <t>Pasa a Disponible</t>
+        </is>
+      </c>
+      <c r="E84" s="46" t="n"/>
+      <c r="F84" s="38" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="G84" s="38" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H84" s="38" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="85" ht="30" customHeight="1" s="43">
+      <c r="A85" s="55" t="n"/>
+      <c r="B85" s="38" t="inlineStr">
+        <is>
+          <t>Regresando sin paciente + SolicitudDeTraslado()</t>
+        </is>
+      </c>
+      <c r="C85" s="46" t="n"/>
+      <c r="D85" s="38" t="inlineStr">
+        <is>
+          <t>Pasa a Trasladando</t>
+        </is>
+      </c>
+      <c r="E85" s="46" t="n"/>
+      <c r="F85" s="38" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="G85" s="38" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H85" s="38" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="86" ht="45" customHeight="1" s="43">
+      <c r="A86" s="55" t="n"/>
+      <c r="B86" s="38" t="inlineStr">
+        <is>
+          <t>Regresando sin paciente + SolicitudDeAtencionDomicilio()</t>
+        </is>
+      </c>
+      <c r="C86" s="46" t="n"/>
+      <c r="D86" s="38" t="inlineStr">
+        <is>
+          <t>Pasa a Atendiendo en domicilio</t>
+        </is>
+      </c>
+      <c r="E86" s="46" t="n"/>
+      <c r="F86" s="38" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="G86" s="38" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H86" s="38" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="87" ht="30" customHeight="1" s="43">
+      <c r="A87" s="55" t="n"/>
+      <c r="B87" s="38" t="inlineStr">
+        <is>
+          <t>En taller + SolicitudMantenimiento()</t>
+        </is>
+      </c>
+      <c r="C87" s="46" t="n"/>
+      <c r="D87" s="38" t="inlineStr">
+        <is>
+          <t>Pasa a Regresando del taller</t>
+        </is>
+      </c>
+      <c r="E87" s="46" t="n"/>
+      <c r="F87" s="38" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="G87" s="38" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H87" s="38" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="88" ht="30" customHeight="1" s="43">
+      <c r="A88" s="55" t="n"/>
+      <c r="B88" s="38" t="inlineStr">
+        <is>
+          <t>En taller + RetornoClinica()</t>
+        </is>
+      </c>
+      <c r="C88" s="46" t="n"/>
+      <c r="D88" s="38" t="inlineStr">
+        <is>
+          <t>Sigue en En taller (no puede retornar)</t>
+        </is>
+      </c>
+      <c r="E88" s="46" t="n"/>
+      <c r="F88" s="38" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="G88" s="38" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H88" s="38" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="89" ht="30" customHeight="1" s="43">
+      <c r="A89" s="55" t="n"/>
+      <c r="B89" s="38" t="inlineStr">
+        <is>
+          <t>Regresando del taller + RetornoClinica()</t>
+        </is>
+      </c>
+      <c r="C89" s="46" t="n"/>
+      <c r="D89" s="38" t="inlineStr">
+        <is>
+          <t>Pasa a Disponible</t>
+        </is>
+      </c>
+      <c r="E89" s="46" t="n"/>
+      <c r="F89" s="38" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="G89" s="38" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H89" s="38" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="90" ht="30" customHeight="1" s="43">
+      <c r="A90" s="50" t="n"/>
+      <c r="B90" s="38" t="inlineStr">
+        <is>
+          <t>Regresando del taller + SolicitudMantenimiento()</t>
+        </is>
+      </c>
+      <c r="C90" s="46" t="n"/>
+      <c r="D90" s="38" t="inlineStr">
+        <is>
+          <t>Sigue en Regresando del taller</t>
+        </is>
+      </c>
+      <c r="E90" s="46" t="n"/>
+      <c r="F90" s="38" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="G90" s="38" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H90" s="38" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="91" ht="15" customHeight="1" s="43">
+      <c r="A91" s="47" t="inlineStr">
+        <is>
+          <t>Clases erróneas</t>
+        </is>
+      </c>
+      <c r="B91" s="38" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="C91" s="46" t="n"/>
+      <c r="D91" s="38" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E91" s="46" t="n"/>
+      <c r="F91" s="38" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G91" s="38" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H91" s="38" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" s="54" t="inlineStr">
+        <is>
+          <t>Tabla de Particiones Concurrencia: exclusion mutua en la ambulancia</t>
+        </is>
+      </c>
+      <c r="B94" s="45" t="n"/>
+      <c r="C94" s="45" t="n"/>
+      <c r="D94" s="45" t="n"/>
+      <c r="E94" s="46" t="n"/>
+    </row>
+    <row r="95">
+      <c r="A95" s="47" t="inlineStr">
+        <is>
+          <t>Condición</t>
+        </is>
+      </c>
+      <c r="B95" s="38" t="inlineStr">
+        <is>
+          <t>Clase correcta</t>
+        </is>
+      </c>
+      <c r="C95" s="38" t="inlineStr">
+        <is>
+          <t>Clase</t>
+        </is>
+      </c>
+      <c r="D95" s="38" t="inlineStr">
+        <is>
+          <t>Clase errónea</t>
+        </is>
+      </c>
+      <c r="E95" s="38" t="inlineStr">
+        <is>
+          <t>Clase</t>
+        </is>
+      </c>
+    </row>
+    <row r="96" ht="30" customHeight="1" s="43">
+      <c r="A96" s="47" t="inlineStr">
+        <is>
+          <t>hilos que piden la ambulancia a la vez</t>
+        </is>
+      </c>
+      <c r="B96" s="38" t="inlineStr">
+        <is>
+          <t>1 hilo</t>
+        </is>
+      </c>
+      <c r="C96" s="38" t="n">
+        <v>1</v>
+      </c>
+      <c r="D96" s="38" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E96" s="38" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="97" ht="30" customHeight="1" s="43">
+      <c r="A97" s="47" t="inlineStr">
+        <is>
+          <t>hilos que piden la ambulancia a la vez</t>
+        </is>
+      </c>
+      <c r="B97" s="38" t="inlineStr">
+        <is>
+          <t>2 o mas hilos (ambulancia libre)</t>
+        </is>
+      </c>
+      <c r="C97" s="38" t="n">
+        <v>2</v>
+      </c>
+      <c r="D97" s="38" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E97" s="38" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" s="47" t="inlineStr">
+        <is>
+          <t>Bateria de pruebas Concurrencia: exclusion mutua en la ambulancia</t>
+        </is>
+      </c>
+      <c r="B99" s="45" t="n"/>
+      <c r="C99" s="45" t="n"/>
+      <c r="D99" s="45" t="n"/>
+      <c r="E99" s="45" t="n"/>
+      <c r="F99" s="45" t="n"/>
+      <c r="G99" s="45" t="n"/>
+      <c r="H99" s="46" t="n"/>
+    </row>
+    <row r="100">
+      <c r="A100" s="47" t="n"/>
+      <c r="B100" s="38" t="inlineStr">
+        <is>
+          <t>Entrada</t>
+        </is>
+      </c>
+      <c r="C100" s="46" t="n"/>
+      <c r="D100" s="38" t="inlineStr">
+        <is>
+          <t>Salida</t>
+        </is>
+      </c>
+      <c r="E100" s="46" t="n"/>
+      <c r="F100" s="38" t="inlineStr">
+        <is>
+          <t>Clases cubiertas</t>
+        </is>
+      </c>
+      <c r="G100" s="38" t="inlineStr">
+        <is>
+          <t>Valores limite</t>
+        </is>
+      </c>
+      <c r="H100" s="38" t="inlineStr">
+        <is>
+          <t>Salidas</t>
+        </is>
+      </c>
+    </row>
+    <row r="101" ht="45" customHeight="1" s="43">
+      <c r="A101" s="47" t="inlineStr">
+        <is>
+          <t>Clases correctas</t>
+        </is>
+      </c>
+      <c r="B101" s="38" t="inlineStr">
+        <is>
+          <t>1 hilo llama atenderDomicilio()</t>
+        </is>
+      </c>
+      <c r="C101" s="46" t="n"/>
+      <c r="D101" s="38" t="inlineStr">
+        <is>
+          <t>El hilo termina; el estado recibe SolicitudDeAtencionDomicilio() una vez</t>
+        </is>
+      </c>
+      <c r="E101" s="46" t="n"/>
+      <c r="F101" s="38" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="G101" s="38" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="H101" s="38" t="inlineStr">
+        <is>
+          <t>1 invocacion</t>
+        </is>
+      </c>
+    </row>
+    <row r="102" ht="75" customHeight="1" s="43">
+      <c r="A102" s="55" t="n"/>
+      <c r="B102" s="38" t="inlineStr">
+        <is>
+          <t>5 hilos llaman atenderDomicilio() a la vez (arrancan juntos con un CountDownLatch)</t>
+        </is>
+      </c>
+      <c r="C102" s="46" t="n"/>
+      <c r="D102" s="38" t="inlineStr">
+        <is>
+          <t>Solo 1 hilo obtiene la ambulancia; los otros 4 quedan esperando (Thread.State WAITING); el estado recibe 1 invocacion</t>
+        </is>
+      </c>
+      <c r="E102" s="46" t="n"/>
+      <c r="F102" s="38" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="G102" s="38" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="H102" s="38" t="inlineStr">
+        <is>
+          <t>1 invocacion, 4 en espera</t>
+        </is>
+      </c>
+    </row>
+    <row r="103" ht="75" customHeight="1" s="43">
+      <c r="A103" s="55" t="n"/>
+      <c r="B103" s="38" t="inlineStr">
+        <is>
+          <t>Los 5 hilos y se libera la ambulancia 4 veces con regresarSinPaciente()</t>
+        </is>
+      </c>
+      <c r="C103" s="46" t="n"/>
+      <c r="D103" s="38" t="inlineStr">
+        <is>
+          <t>Los 5 hilos terminan; nunca hay mas de 1 hilo dentro a la vez; 5 invocaciones en total; sin deadlock (timeout)</t>
+        </is>
+      </c>
+      <c r="E103" s="46" t="n"/>
+      <c r="F103" s="38" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="G103" s="38" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="H103" s="38" t="inlineStr">
+        <is>
+          <t>5 invocaciones</t>
+        </is>
+      </c>
+    </row>
+    <row r="104" ht="60" customHeight="1" s="43">
+      <c r="A104" s="50" t="n"/>
+      <c r="B104" s="38" t="inlineStr">
+        <is>
+          <t>1 operario (solicitarMantenimiento) y 1 asociado (atenderDomicilio) a la vez</t>
+        </is>
+      </c>
+      <c r="C104" s="46" t="n"/>
+      <c r="D104" s="38" t="inlineStr">
+        <is>
+          <t>Solo uno obtiene la ambulancia primero; el otro espera y termina al liberarse; sin deadlock</t>
+        </is>
+      </c>
+      <c r="E104" s="46" t="n"/>
+      <c r="F104" s="38" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="G104" s="38" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="H104" s="38" t="inlineStr">
+        <is>
+          <t>1 espera</t>
+        </is>
+      </c>
+    </row>
+    <row r="105" ht="15" customHeight="1" s="43">
+      <c r="A105" s="47" t="inlineStr">
+        <is>
+          <t>Clases erróneas</t>
+        </is>
+      </c>
+      <c r="B105" s="38" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="C105" s="46" t="n"/>
+      <c r="D105" s="38" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E105" s="46" t="n"/>
+      <c r="F105" s="38" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G105" s="38" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H105" s="38" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" s="54" t="inlineStr">
+        <is>
+          <t>Tabla de Particiones Concurrencia: espera, despertar e interrupcion</t>
+        </is>
+      </c>
+      <c r="B108" s="45" t="n"/>
+      <c r="C108" s="45" t="n"/>
+      <c r="D108" s="45" t="n"/>
+      <c r="E108" s="46" t="n"/>
+    </row>
+    <row r="109">
+      <c r="A109" s="47" t="inlineStr">
+        <is>
+          <t>Condición</t>
+        </is>
+      </c>
+      <c r="B109" s="38" t="inlineStr">
+        <is>
+          <t>Clase correcta</t>
+        </is>
+      </c>
+      <c r="C109" s="38" t="inlineStr">
+        <is>
+          <t>Clase</t>
+        </is>
+      </c>
+      <c r="D109" s="38" t="inlineStr">
+        <is>
+          <t>Clase errónea</t>
+        </is>
+      </c>
+      <c r="E109" s="38" t="inlineStr">
+        <is>
+          <t>Clase</t>
+        </is>
+      </c>
+    </row>
+    <row r="110" ht="30" customHeight="1" s="43">
+      <c r="A110" s="47" t="inlineStr">
+        <is>
+          <t>ambulancia</t>
+        </is>
+      </c>
+      <c r="B110" s="38" t="inlineStr">
+        <is>
+          <t>Ocupada y simulacion activa</t>
+        </is>
+      </c>
+      <c r="C110" s="38" t="n">
+        <v>1</v>
+      </c>
+      <c r="D110" s="38" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E110" s="38" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="111" ht="30" customHeight="1" s="43">
+      <c r="A111" s="47" t="inlineStr">
+        <is>
+          <t>evento</t>
+        </is>
+      </c>
+      <c r="B111" s="38" t="inlineStr">
+        <is>
+          <t>Se libera la ambulancia (notifyAll)</t>
+        </is>
+      </c>
+      <c r="C111" s="38" t="n">
+        <v>2</v>
+      </c>
+      <c r="D111" s="38" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E111" s="38" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="112" ht="30" customHeight="1" s="43">
+      <c r="A112" s="47" t="inlineStr">
+        <is>
+          <t>evento</t>
+        </is>
+      </c>
+      <c r="B112" s="38" t="inlineStr">
+        <is>
+          <t>Termina la simulacion (setSimulacionActiva(false))</t>
+        </is>
+      </c>
+      <c r="C112" s="38" t="n">
+        <v>3</v>
+      </c>
+      <c r="D112" s="38" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E112" s="38" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="113" ht="30" customHeight="1" s="43">
+      <c r="A113" s="47" t="inlineStr">
+        <is>
+          <t>evento</t>
+        </is>
+      </c>
+      <c r="B113" s="38" t="inlineStr">
+        <is>
+          <t>Se interrumpe el hilo que espera</t>
+        </is>
+      </c>
+      <c r="C113" s="38" t="n">
+        <v>4</v>
+      </c>
+      <c r="D113" s="38" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E113" s="38" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" s="47" t="inlineStr">
+        <is>
+          <t>Bateria de pruebas Concurrencia: espera, despertar e interrupcion</t>
+        </is>
+      </c>
+      <c r="B115" s="45" t="n"/>
+      <c r="C115" s="45" t="n"/>
+      <c r="D115" s="45" t="n"/>
+      <c r="E115" s="45" t="n"/>
+      <c r="F115" s="45" t="n"/>
+      <c r="G115" s="45" t="n"/>
+      <c r="H115" s="46" t="n"/>
+    </row>
+    <row r="116">
+      <c r="A116" s="47" t="n"/>
+      <c r="B116" s="38" t="inlineStr">
+        <is>
+          <t>Entrada</t>
+        </is>
+      </c>
+      <c r="C116" s="46" t="n"/>
+      <c r="D116" s="38" t="inlineStr">
+        <is>
+          <t>Salida</t>
+        </is>
+      </c>
+      <c r="E116" s="46" t="n"/>
+      <c r="F116" s="38" t="inlineStr">
+        <is>
+          <t>Clases cubiertas</t>
+        </is>
+      </c>
+      <c r="G116" s="38" t="inlineStr">
+        <is>
+          <t>Valores limite</t>
+        </is>
+      </c>
+      <c r="H116" s="38" t="inlineStr">
+        <is>
+          <t>Salidas</t>
+        </is>
+      </c>
+    </row>
+    <row r="117" ht="45" customHeight="1" s="43">
+      <c r="A117" s="47" t="inlineStr">
+        <is>
+          <t>Clases correctas</t>
+        </is>
+      </c>
+      <c r="B117" s="38" t="inlineStr">
+        <is>
+          <t>Hilo llama atenderDomicilio() con la ambulancia ocupada</t>
+        </is>
+      </c>
+      <c r="C117" s="46" t="n"/>
+      <c r="D117" s="38" t="inlineStr">
+        <is>
+          <t>El hilo queda esperando (WAITING)</t>
+        </is>
+      </c>
+      <c r="E117" s="46" t="n"/>
+      <c r="F117" s="38" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="G117" s="38" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H117" s="38" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="118" ht="75" customHeight="1" s="43">
+      <c r="A118" s="55" t="n"/>
+      <c r="B118" s="38" t="inlineStr">
+        <is>
+          <t>Con el hilo esperando, otro hilo llama regresarSinPaciente()</t>
+        </is>
+      </c>
+      <c r="C118" s="46" t="n"/>
+      <c r="D118" s="38" t="inlineStr">
+        <is>
+          <t>El hilo en espera se despierta, toma la ambulancia y termina (estado recibe SolicitudDeAtencionDomicilio())</t>
+        </is>
+      </c>
+      <c r="E118" s="46" t="n"/>
+      <c r="F118" s="38" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="G118" s="38" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H118" s="38" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="119" ht="45" customHeight="1" s="43">
+      <c r="A119" s="55" t="n"/>
+      <c r="B119" s="38" t="inlineStr">
+        <is>
+          <t>Con 3 hilos esperando, otro hilo llama setSimulacionActiva(false)</t>
+        </is>
+      </c>
+      <c r="C119" s="46" t="n"/>
+      <c r="D119" s="38" t="inlineStr">
+        <is>
+          <t>Los 3 hilos se despiertan y terminan sin invocar al estado</t>
+        </is>
+      </c>
+      <c r="E119" s="46" t="n"/>
+      <c r="F119" s="38" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="G119" s="38" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="H119" s="38" t="inlineStr">
+        <is>
+          <t>0 invocaciones</t>
+        </is>
+      </c>
+    </row>
+    <row r="120" ht="60" customHeight="1" s="43">
+      <c r="A120" s="50" t="n"/>
+      <c r="B120" s="38" t="inlineStr">
+        <is>
+          <t>Con el hilo esperando, se llama interrupt() sobre el hilo</t>
+        </is>
+      </c>
+      <c r="C120" s="46" t="n"/>
+      <c r="D120" s="38" t="inlineStr">
+        <is>
+          <t>El hilo termina; su bandera de interrupcion queda activada; el estado no cambia</t>
+        </is>
+      </c>
+      <c r="E120" s="46" t="n"/>
+      <c r="F120" s="38" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="G120" s="38" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H120" s="38" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="121" ht="15" customHeight="1" s="43">
+      <c r="A121" s="47" t="inlineStr">
+        <is>
+          <t>Clases erróneas</t>
+        </is>
+      </c>
+      <c r="B121" s="38" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="C121" s="46" t="n"/>
+      <c r="D121" s="38" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E121" s="46" t="n"/>
+      <c r="F121" s="38" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G121" s="38" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H121" s="38" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" s="54" t="inlineStr">
+        <is>
+          <t>Tabla de Particiones RetornoAutomatico (hilo)</t>
+        </is>
+      </c>
+      <c r="B124" s="45" t="n"/>
+      <c r="C124" s="45" t="n"/>
+      <c r="D124" s="45" t="n"/>
+      <c r="E124" s="46" t="n"/>
+    </row>
+    <row r="125">
+      <c r="A125" s="47" t="inlineStr">
+        <is>
+          <t>Condición</t>
+        </is>
+      </c>
+      <c r="B125" s="38" t="inlineStr">
+        <is>
+          <t>Clase correcta</t>
+        </is>
+      </c>
+      <c r="C125" s="38" t="inlineStr">
+        <is>
+          <t>Clase</t>
+        </is>
+      </c>
+      <c r="D125" s="38" t="inlineStr">
+        <is>
+          <t>Clase errónea</t>
+        </is>
+      </c>
+      <c r="E125" s="38" t="inlineStr">
+        <is>
+          <t>Clase</t>
+        </is>
+      </c>
+    </row>
+    <row r="126" ht="15" customHeight="1" s="43">
+      <c r="A126" s="47" t="inlineStr">
+        <is>
+          <t>simulacion</t>
+        </is>
+      </c>
+      <c r="B126" s="38" t="inlineStr">
+        <is>
+          <t>Activa</t>
+        </is>
+      </c>
+      <c r="C126" s="38" t="n">
+        <v>1</v>
+      </c>
+      <c r="D126" s="38" t="inlineStr">
+        <is>
+          <t>Finalizada</t>
+        </is>
+      </c>
+      <c r="E126" s="38" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="127" ht="30" customHeight="1" s="43">
+      <c r="A127" s="47" t="inlineStr">
+        <is>
+          <t>hilo</t>
+        </is>
+      </c>
+      <c r="B127" s="38" t="inlineStr">
+        <is>
+          <t>Interrumpido mientras duerme</t>
+        </is>
+      </c>
+      <c r="C127" s="38" t="n">
+        <v>3</v>
+      </c>
+      <c r="D127" s="38" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E127" s="38" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" s="47" t="inlineStr">
+        <is>
+          <t>Bateria de pruebas RetornoAutomatico (hilo)</t>
+        </is>
+      </c>
+      <c r="B129" s="45" t="n"/>
+      <c r="C129" s="45" t="n"/>
+      <c r="D129" s="45" t="n"/>
+      <c r="E129" s="45" t="n"/>
+      <c r="F129" s="45" t="n"/>
+      <c r="G129" s="45" t="n"/>
+      <c r="H129" s="46" t="n"/>
+    </row>
+    <row r="130">
+      <c r="A130" s="47" t="n"/>
+      <c r="B130" s="38" t="inlineStr">
+        <is>
+          <t>Entrada</t>
+        </is>
+      </c>
+      <c r="C130" s="46" t="n"/>
+      <c r="D130" s="38" t="inlineStr">
+        <is>
+          <t>Salida</t>
+        </is>
+      </c>
+      <c r="E130" s="46" t="n"/>
+      <c r="F130" s="38" t="inlineStr">
+        <is>
+          <t>Clases cubiertas</t>
+        </is>
+      </c>
+      <c r="G130" s="38" t="inlineStr">
+        <is>
+          <t>Valores limite</t>
+        </is>
+      </c>
+      <c r="H130" s="38" t="inlineStr">
+        <is>
+          <t>Salidas</t>
+        </is>
+      </c>
+    </row>
+    <row r="131" ht="45" customHeight="1" s="43">
+      <c r="A131" s="47" t="inlineStr">
+        <is>
+          <t>Clases correctas</t>
+        </is>
+      </c>
+      <c r="B131" s="38" t="inlineStr">
+        <is>
+          <t>Hilo RetornoAutomatico con simulacion activa; se lo observa 500 ms</t>
+        </is>
+      </c>
+      <c r="C131" s="46" t="n"/>
+      <c r="D131" s="38" t="inlineStr">
+        <is>
+          <t>El hilo sigue vivo (durmiendo hasta su proximo intento)</t>
+        </is>
+      </c>
+      <c r="E131" s="46" t="n"/>
+      <c r="F131" s="38" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="G131" s="38" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H131" s="38" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="132" ht="45" customHeight="1" s="43">
+      <c r="A132" s="50" t="n"/>
+      <c r="B132" s="38" t="inlineStr">
+        <is>
+          <t>Hilo RetornoAutomatico dormido; se llama interrupt()</t>
+        </is>
+      </c>
+      <c r="C132" s="46" t="n"/>
+      <c r="D132" s="38" t="inlineStr">
+        <is>
+          <t>El hilo termina limpiamente (isAlive() falso) en menos de 1 s</t>
+        </is>
+      </c>
+      <c r="E132" s="46" t="n"/>
+      <c r="F132" s="38" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="G132" s="38" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H132" s="38" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="133" ht="45" customHeight="1" s="43">
+      <c r="A133" s="47" t="inlineStr">
+        <is>
+          <t>Clases erróneas</t>
+        </is>
+      </c>
+      <c r="B133" s="38" t="inlineStr">
+        <is>
+          <t>Hilo RetornoAutomatico con simulacion ya finalizada</t>
+        </is>
+      </c>
+      <c r="C133" s="46" t="n"/>
+      <c r="D133" s="38" t="inlineStr">
+        <is>
+          <t>El hilo termina de inmediato (menos de 1 s) sin invocar retornoAutomatico</t>
+        </is>
+      </c>
+      <c r="E133" s="46" t="n"/>
+      <c r="F133" s="38" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="G133" s="38" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H133" s="38" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="138">
+    <mergeCell ref="B91:C91"/>
+    <mergeCell ref="D20:E20"/>
+    <mergeCell ref="A39:E39"/>
+    <mergeCell ref="D60:E60"/>
+    <mergeCell ref="B100:C100"/>
+    <mergeCell ref="D100:E100"/>
+    <mergeCell ref="A20:A22"/>
+    <mergeCell ref="A11:E11"/>
+    <mergeCell ref="B22:C22"/>
+    <mergeCell ref="A1:E1"/>
+    <mergeCell ref="D84:E84"/>
+    <mergeCell ref="D22:E22"/>
+    <mergeCell ref="A94:E94"/>
+    <mergeCell ref="D36:E36"/>
+    <mergeCell ref="B102:C102"/>
+    <mergeCell ref="B77:C77"/>
+    <mergeCell ref="D6:E6"/>
+    <mergeCell ref="B21:C21"/>
+    <mergeCell ref="D77:E77"/>
+    <mergeCell ref="A65:E65"/>
+    <mergeCell ref="B86:C86"/>
+    <mergeCell ref="D86:E86"/>
+    <mergeCell ref="B61:C61"/>
+    <mergeCell ref="B101:C101"/>
+    <mergeCell ref="D61:E61"/>
+    <mergeCell ref="D48:E48"/>
+    <mergeCell ref="B78:C78"/>
+    <mergeCell ref="D7:E7"/>
+    <mergeCell ref="D78:E78"/>
+    <mergeCell ref="D62:E62"/>
+    <mergeCell ref="A5:H5"/>
+    <mergeCell ref="B49:C49"/>
+    <mergeCell ref="B33:C33"/>
+    <mergeCell ref="B104:C104"/>
+    <mergeCell ref="D33:E33"/>
+    <mergeCell ref="B32:C32"/>
+    <mergeCell ref="D88:E88"/>
+    <mergeCell ref="B35:C35"/>
+    <mergeCell ref="A31:H31"/>
+    <mergeCell ref="D35:E35"/>
+    <mergeCell ref="A117:A120"/>
+    <mergeCell ref="B90:C90"/>
+    <mergeCell ref="D19:E19"/>
+    <mergeCell ref="D34:E34"/>
+    <mergeCell ref="D90:E90"/>
+    <mergeCell ref="B131:C131"/>
+    <mergeCell ref="D131:E131"/>
+    <mergeCell ref="B18:C18"/>
+    <mergeCell ref="D101:E101"/>
+    <mergeCell ref="B130:C130"/>
+    <mergeCell ref="B117:C117"/>
+    <mergeCell ref="D76:E76"/>
+    <mergeCell ref="A99:H99"/>
+    <mergeCell ref="D132:E132"/>
+    <mergeCell ref="B132:C132"/>
+    <mergeCell ref="D75:E75"/>
+    <mergeCell ref="B119:C119"/>
+    <mergeCell ref="D47:E47"/>
+    <mergeCell ref="B116:C116"/>
+    <mergeCell ref="A131:A132"/>
+    <mergeCell ref="B103:C103"/>
+    <mergeCell ref="D103:E103"/>
+    <mergeCell ref="A76:A90"/>
+    <mergeCell ref="B84:C84"/>
+    <mergeCell ref="B118:C118"/>
+    <mergeCell ref="D118:E118"/>
+    <mergeCell ref="B6:C6"/>
+    <mergeCell ref="B80:C80"/>
+    <mergeCell ref="B89:C89"/>
+    <mergeCell ref="D89:E89"/>
+    <mergeCell ref="B79:C79"/>
+    <mergeCell ref="D79:E79"/>
+    <mergeCell ref="B7:C7"/>
+    <mergeCell ref="B81:C81"/>
+    <mergeCell ref="D81:E81"/>
+    <mergeCell ref="B121:C121"/>
+    <mergeCell ref="B105:C105"/>
+    <mergeCell ref="B58:C58"/>
+    <mergeCell ref="D105:E105"/>
+    <mergeCell ref="A124:E124"/>
+    <mergeCell ref="A59:A61"/>
+    <mergeCell ref="A34:A36"/>
+    <mergeCell ref="D49:E49"/>
+    <mergeCell ref="A25:E25"/>
+    <mergeCell ref="B120:C120"/>
+    <mergeCell ref="D120:E120"/>
+    <mergeCell ref="A108:E108"/>
+    <mergeCell ref="B60:C60"/>
+    <mergeCell ref="D116:E116"/>
+    <mergeCell ref="B88:C88"/>
+    <mergeCell ref="B82:C82"/>
+    <mergeCell ref="A74:H74"/>
+    <mergeCell ref="D91:E91"/>
+    <mergeCell ref="A101:A104"/>
+    <mergeCell ref="B19:C19"/>
+    <mergeCell ref="B34:C34"/>
+    <mergeCell ref="A129:H129"/>
+    <mergeCell ref="D102:E102"/>
+    <mergeCell ref="B83:C83"/>
+    <mergeCell ref="A17:H17"/>
+    <mergeCell ref="D83:E83"/>
+    <mergeCell ref="D117:E117"/>
+    <mergeCell ref="B20:C20"/>
+    <mergeCell ref="B76:C76"/>
+    <mergeCell ref="B133:C133"/>
+    <mergeCell ref="D133:E133"/>
+    <mergeCell ref="A115:H115"/>
+    <mergeCell ref="B85:C85"/>
+    <mergeCell ref="D85:E85"/>
+    <mergeCell ref="B75:C75"/>
+    <mergeCell ref="B47:C47"/>
+    <mergeCell ref="B62:C62"/>
+    <mergeCell ref="B59:C59"/>
+    <mergeCell ref="D119:E119"/>
+    <mergeCell ref="B46:C46"/>
+    <mergeCell ref="D46:E46"/>
+    <mergeCell ref="A45:H45"/>
+    <mergeCell ref="D80:E80"/>
+    <mergeCell ref="D21:E21"/>
+    <mergeCell ref="B48:C48"/>
+    <mergeCell ref="D104:E104"/>
+    <mergeCell ref="D32:E32"/>
+    <mergeCell ref="B8:C8"/>
+    <mergeCell ref="B87:C87"/>
+    <mergeCell ref="D87:E87"/>
+    <mergeCell ref="A48:A50"/>
+    <mergeCell ref="A57:H57"/>
+    <mergeCell ref="D18:E18"/>
+    <mergeCell ref="D58:E58"/>
+    <mergeCell ref="D8:E8"/>
+    <mergeCell ref="A53:E53"/>
+    <mergeCell ref="D121:E121"/>
+    <mergeCell ref="D130:E130"/>
+    <mergeCell ref="D82:E82"/>
+    <mergeCell ref="B36:C36"/>
+    <mergeCell ref="B50:C50"/>
+    <mergeCell ref="D50:E50"/>
+    <mergeCell ref="D59:E59"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>